<commit_message>
Ekatte/Milestone-20260111/Task- 86c7fc2vh - Add statistics export to the data file, refactor code, and add unit tests for sorting handler
</commit_message>
<xml_diff>
--- a/Ekatteproject/export/statistics.xlsx
+++ b/Ekatteproject/export/statistics.xlsx
@@ -5,33 +5,58 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="Statistics" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Export Stats" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
-  <si>
-    <t>id</t>
-  </si>
-  <si>
-    <t>name</t>
-  </si>
-  <si>
-    <t>name_en</t>
-  </si>
-  <si>
-    <t>Village1</t>
-  </si>
-  <si>
-    <t>Village1EN</t>
-  </si>
-  <si>
-    <t>Village2</t>
-  </si>
-  <si>
-    <t>Village2EN</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+  <si>
+    <t>Table</t>
+  </si>
+  <si>
+    <t>Count rows</t>
+  </si>
+  <si>
+    <t>village_count</t>
+  </si>
+  <si>
+    <t>166</t>
+  </si>
+  <si>
+    <t>district_count</t>
+  </si>
+  <si>
+    <t>28</t>
+  </si>
+  <si>
+    <t>township_count</t>
+  </si>
+  <si>
+    <t>265</t>
+  </si>
+  <si>
+    <t>cityhalls_count</t>
+  </si>
+  <si>
+    <t>3155</t>
+  </si>
+  <si>
+    <t>Execution time (ms)</t>
+  </si>
+  <si>
+    <t>Memory used (MB)</t>
+  </si>
+  <si>
+    <t>0.04</t>
+  </si>
+  <si>
+    <t>CPU used (ms)</t>
+  </si>
+  <si>
+    <t>0.00</t>
   </si>
 </sst>
 </file>
@@ -408,40 +433,82 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>1</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>
       </c>
-      <c r="C2" t="s">
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>2</v>
       </c>
       <c r="B3" t="s">
         <v>5</v>
       </c>
-      <c r="C3" t="s">
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1">
+        <v>6.3572</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ekatte/Milestone-20260118/Task- 86c7fc2vh - Add supertest library for integration test on the controllers. Refactored the code and added more unit-test
</commit_message>
<xml_diff>
--- a/Ekatteproject/export/statistics.xlsx
+++ b/Ekatteproject/export/statistics.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>Table</t>
   </si>
@@ -23,7 +23,7 @@
     <t>village_count</t>
   </si>
   <si>
-    <t>166</t>
+    <t>165</t>
   </si>
   <si>
     <t>district_count</t>
@@ -44,19 +44,22 @@
     <t>3155</t>
   </si>
   <si>
+    <t>--- EXPORT STATISTICS ---</t>
+  </si>
+  <si>
     <t>Execution time (ms)</t>
   </si>
   <si>
     <t>Memory used (MB)</t>
   </si>
   <si>
-    <t>0.04</t>
+    <t>0.11</t>
   </si>
   <si>
     <t>CPU used (ms)</t>
   </si>
   <si>
-    <t>0.00</t>
+    <t>968.00</t>
   </si>
 </sst>
 </file>
@@ -484,31 +487,36 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>10</v>
-      </c>
-      <c r="B1">
-        <v>6.3572</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>11</v>
       </c>
-      <c r="B2" t="s">
-        <v>12</v>
+      <c r="B2">
+        <v>5.4965</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" t="s">
         <v>13</v>
       </c>
-      <c r="B3" t="s">
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>14</v>
+      </c>
+      <c r="B4" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>